<commit_message>
Enhanced the isotherm file layout
</commit_message>
<xml_diff>
--- a/src/reactormodels/IO/data/experimental_input_isotherm.xlsx
+++ b/src/reactormodels/IO/data/experimental_input_isotherm.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mohammedfaran/Desktop/Research Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{199F0933-023D-BA4F-AE19-7D072BC0F71B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62732C09-E956-CA4B-864F-D0EA261BECF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8240" yWindow="500" windowWidth="27860" windowHeight="17500" xr2:uid="{FB75EC0D-8373-7F4F-A4DF-7E2B42744032}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{FB75EC0D-8373-7F4F-A4DF-7E2B42744032}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="181029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="36">
   <si>
     <t>K</t>
   </si>
@@ -142,13 +141,16 @@
   </si>
   <si>
     <t>NBP1</t>
+  </si>
+  <si>
+    <t>time</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -170,12 +172,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -189,7 +185,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -202,8 +198,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -226,19 +228,96 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -573,415 +652,846 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{343F2F1A-4C43-6844-A4B4-CF0DBA1765B6}">
-  <dimension ref="A1:AA18"/>
+  <dimension ref="A1:BA16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" customWidth="1"/>
+    <col min="7" max="7" width="11.6640625" customWidth="1"/>
+    <col min="9" max="27" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:53" x14ac:dyDescent="0.2">
+      <c r="A1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="11"/>
+      <c r="D1" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="E1" s="11"/>
+      <c r="F1" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="G1" s="11"/>
+      <c r="H1" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="I1" s="11"/>
+      <c r="J1" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="K1" s="11"/>
+      <c r="L1" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="M1" s="11"/>
+      <c r="N1" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="O1" s="11"/>
+      <c r="P1" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="Q1" s="11"/>
+      <c r="R1" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="S1" s="11"/>
+      <c r="T1" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="L1" s="7" t="s">
+      <c r="U1" s="11"/>
+      <c r="V1" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="M1" s="7" t="s">
+      <c r="W1" s="11"/>
+      <c r="X1" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="N1" s="7" t="s">
+      <c r="Y1" s="11"/>
+      <c r="Z1" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="O1" s="7" t="s">
+      <c r="AA1" s="11"/>
+      <c r="AB1" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="P1" s="7" t="s">
+      <c r="AC1" s="13"/>
+      <c r="AD1" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="Q1" s="7" t="s">
+      <c r="AE1" s="13"/>
+      <c r="AF1" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="R1" s="7" t="s">
+      <c r="AG1" s="13"/>
+      <c r="AH1" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="S1" s="7" t="s">
+      <c r="AI1" s="13"/>
+      <c r="AJ1" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="T1" s="7" t="s">
+      <c r="AK1" s="13"/>
+      <c r="AL1" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="U1" s="7" t="s">
+      <c r="AM1" s="13"/>
+      <c r="AN1" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="V1" s="7" t="s">
+      <c r="AO1" s="13"/>
+      <c r="AP1" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="W1" s="7" t="s">
+      <c r="AQ1" s="13"/>
+      <c r="AR1" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="X1" s="7" t="s">
+      <c r="AS1" s="13"/>
+      <c r="AT1" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="Y1" s="7" t="s">
+      <c r="AU1" s="13"/>
+      <c r="AV1" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="Z1" s="7" t="s">
+      <c r="AW1" s="13"/>
+      <c r="AX1" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="AA1" s="3" t="s">
+      <c r="AY1" s="13"/>
+      <c r="AZ1" s="14" t="s">
         <v>34</v>
       </c>
+      <c r="BA1" s="15"/>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:53" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
+      <c r="C2" s="7"/>
       <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
+      <c r="E2" s="7"/>
       <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
+      <c r="G2" s="7"/>
       <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6"/>
-      <c r="N2" s="6"/>
-      <c r="O2" s="6"/>
-      <c r="P2" s="6"/>
-      <c r="Q2" s="6"/>
-      <c r="R2" s="6"/>
-      <c r="S2" s="6"/>
-      <c r="T2" s="6"/>
-      <c r="U2" s="6"/>
-      <c r="V2" s="6"/>
-      <c r="W2" s="6"/>
-      <c r="X2" s="6"/>
-      <c r="Y2" s="6"/>
-      <c r="Z2" s="6"/>
-      <c r="AA2" s="6"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
+      <c r="K2" s="7"/>
+      <c r="L2" s="7"/>
+      <c r="M2" s="7"/>
+      <c r="N2" s="7"/>
+      <c r="O2" s="7"/>
+      <c r="P2" s="7"/>
+      <c r="Q2" s="7"/>
+      <c r="R2" s="7"/>
+      <c r="S2" s="7"/>
+      <c r="T2" s="7"/>
+      <c r="U2" s="7"/>
+      <c r="V2" s="7"/>
+      <c r="W2" s="7"/>
+      <c r="X2" s="7"/>
+      <c r="Y2" s="7"/>
+      <c r="Z2" s="7"/>
+      <c r="AA2" s="7"/>
+      <c r="AB2" s="6"/>
+      <c r="AC2" s="6"/>
+      <c r="AD2" s="6"/>
+      <c r="AE2" s="6"/>
+      <c r="AF2" s="6"/>
+      <c r="AG2" s="6"/>
+      <c r="AH2" s="6"/>
+      <c r="AI2" s="6"/>
+      <c r="AJ2" s="6"/>
+      <c r="AK2" s="6"/>
+      <c r="AL2" s="6"/>
+      <c r="AM2" s="6"/>
+      <c r="AN2" s="6"/>
+      <c r="AO2" s="6"/>
+      <c r="AP2" s="6"/>
+      <c r="AQ2" s="6"/>
+      <c r="AR2" s="6"/>
+      <c r="AS2" s="6"/>
+      <c r="AT2" s="6"/>
+      <c r="AU2" s="6"/>
+      <c r="AV2" s="6"/>
+      <c r="AW2" s="6"/>
+      <c r="AX2" s="6"/>
+      <c r="AY2" s="6"/>
+      <c r="AZ2" s="6"/>
+      <c r="BA2" s="6"/>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
-        <v>6</v>
+    <row r="3" spans="1:53" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>0</v>
       </c>
       <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
+      <c r="C3" s="8"/>
       <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
+      <c r="E3" s="8"/>
       <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
+      <c r="G3" s="8"/>
       <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6"/>
-      <c r="M3" s="6"/>
-      <c r="N3" s="6"/>
-      <c r="O3" s="6"/>
-      <c r="P3" s="6"/>
-      <c r="Q3" s="6"/>
-      <c r="R3" s="6"/>
-      <c r="S3" s="6"/>
-      <c r="T3" s="6"/>
-      <c r="U3" s="6"/>
-      <c r="V3" s="6"/>
-      <c r="W3" s="6"/>
-      <c r="X3" s="6"/>
-      <c r="Y3" s="6"/>
-      <c r="Z3" s="6"/>
-      <c r="AA3" s="6"/>
+      <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+      <c r="L3" s="8"/>
+      <c r="M3" s="8"/>
+      <c r="N3" s="8"/>
+      <c r="O3" s="8"/>
+      <c r="P3" s="8"/>
+      <c r="Q3" s="8"/>
+      <c r="R3" s="8"/>
+      <c r="S3" s="8"/>
+      <c r="T3" s="8"/>
+      <c r="U3" s="8"/>
+      <c r="V3" s="8"/>
+      <c r="W3" s="8"/>
+      <c r="X3" s="8"/>
+      <c r="Y3" s="8"/>
+      <c r="Z3" s="8"/>
+      <c r="AA3" s="8"/>
+      <c r="AB3" s="6"/>
+      <c r="AC3" s="6"/>
+      <c r="AD3" s="6"/>
+      <c r="AE3" s="6"/>
+      <c r="AF3" s="6"/>
+      <c r="AG3" s="6"/>
+      <c r="AH3" s="6"/>
+      <c r="AI3" s="6"/>
+      <c r="AJ3" s="6"/>
+      <c r="AK3" s="6"/>
+      <c r="AL3" s="6"/>
+      <c r="AM3" s="6"/>
+      <c r="AN3" s="6"/>
+      <c r="AO3" s="6"/>
+      <c r="AP3" s="6"/>
+      <c r="AQ3" s="6"/>
+      <c r="AR3" s="6"/>
+      <c r="AS3" s="6"/>
+      <c r="AT3" s="6"/>
+      <c r="AU3" s="6"/>
+      <c r="AV3" s="6"/>
+      <c r="AW3" s="6"/>
+      <c r="AX3" s="6"/>
+      <c r="AY3" s="6"/>
+      <c r="AZ3" s="6"/>
+      <c r="BA3" s="6"/>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
-        <v>7</v>
+    <row r="4" spans="1:53" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>3</v>
       </c>
       <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
+      <c r="C4" s="7"/>
       <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
+      <c r="E4" s="7"/>
       <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
+      <c r="G4" s="7"/>
       <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
-      <c r="K4" s="6"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="6"/>
-      <c r="N4" s="6"/>
-      <c r="O4" s="6"/>
-      <c r="P4" s="6"/>
-      <c r="Q4" s="6"/>
-      <c r="R4" s="6"/>
-      <c r="S4" s="6"/>
-      <c r="T4" s="6"/>
-      <c r="U4" s="6"/>
-      <c r="V4" s="6"/>
-      <c r="W4" s="6"/>
-      <c r="X4" s="6"/>
-      <c r="Y4" s="6"/>
-      <c r="Z4" s="6"/>
-      <c r="AA4" s="6"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="7"/>
+      <c r="M4" s="7"/>
+      <c r="N4" s="7"/>
+      <c r="O4" s="7"/>
+      <c r="P4" s="7"/>
+      <c r="Q4" s="7"/>
+      <c r="R4" s="7"/>
+      <c r="S4" s="7"/>
+      <c r="T4" s="7"/>
+      <c r="U4" s="7"/>
+      <c r="V4" s="7"/>
+      <c r="W4" s="7"/>
+      <c r="X4" s="7"/>
+      <c r="Y4" s="7"/>
+      <c r="Z4" s="7"/>
+      <c r="AA4" s="7"/>
+      <c r="AB4" s="6"/>
+      <c r="AC4" s="6"/>
+      <c r="AD4" s="6"/>
+      <c r="AE4" s="6"/>
+      <c r="AF4" s="6"/>
+      <c r="AG4" s="6"/>
+      <c r="AH4" s="6"/>
+      <c r="AI4" s="6"/>
+      <c r="AJ4" s="6"/>
+      <c r="AK4" s="6"/>
+      <c r="AL4" s="6"/>
+      <c r="AM4" s="6"/>
+      <c r="AN4" s="6"/>
+      <c r="AO4" s="6"/>
+      <c r="AP4" s="6"/>
+      <c r="AQ4" s="6"/>
+      <c r="AR4" s="6"/>
+      <c r="AS4" s="6"/>
+      <c r="AT4" s="6"/>
+      <c r="AU4" s="6"/>
+      <c r="AV4" s="6"/>
+      <c r="AW4" s="6"/>
+      <c r="AX4" s="6"/>
+      <c r="AY4" s="6"/>
+      <c r="AZ4" s="6"/>
+      <c r="BA4" s="6"/>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A5" s="4" t="s">
+    <row r="5" spans="1:53" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
+      <c r="C5" s="8"/>
       <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
+      <c r="E5" s="8"/>
       <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
+      <c r="G5" s="8"/>
       <c r="H5" s="6"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6"/>
-      <c r="K5" s="6"/>
-      <c r="L5" s="6"/>
-      <c r="M5" s="6"/>
-      <c r="N5" s="6"/>
-      <c r="O5" s="6"/>
-      <c r="P5" s="6"/>
-      <c r="Q5" s="6"/>
-      <c r="R5" s="6"/>
-      <c r="S5" s="6"/>
-      <c r="T5" s="6"/>
-      <c r="U5" s="6"/>
-      <c r="V5" s="6"/>
-      <c r="W5" s="6"/>
-      <c r="X5" s="6"/>
-      <c r="Y5" s="6"/>
-      <c r="Z5" s="6"/>
-      <c r="AA5" s="6"/>
+      <c r="I5" s="8"/>
+      <c r="J5" s="8"/>
+      <c r="K5" s="8"/>
+      <c r="L5" s="8"/>
+      <c r="M5" s="8"/>
+      <c r="N5" s="8"/>
+      <c r="O5" s="8"/>
+      <c r="P5" s="8"/>
+      <c r="Q5" s="8"/>
+      <c r="R5" s="8"/>
+      <c r="S5" s="8"/>
+      <c r="T5" s="8"/>
+      <c r="U5" s="8"/>
+      <c r="V5" s="8"/>
+      <c r="W5" s="8"/>
+      <c r="X5" s="8"/>
+      <c r="Y5" s="8"/>
+      <c r="Z5" s="8"/>
+      <c r="AA5" s="8"/>
+      <c r="AB5" s="6"/>
+      <c r="AC5" s="6"/>
+      <c r="AD5" s="6"/>
+      <c r="AE5" s="6"/>
+      <c r="AF5" s="6"/>
+      <c r="AG5" s="6"/>
+      <c r="AH5" s="6"/>
+      <c r="AI5" s="6"/>
+      <c r="AJ5" s="6"/>
+      <c r="AK5" s="6"/>
+      <c r="AL5" s="6"/>
+      <c r="AM5" s="6"/>
+      <c r="AN5" s="6"/>
+      <c r="AO5" s="6"/>
+      <c r="AP5" s="6"/>
+      <c r="AQ5" s="6"/>
+      <c r="AR5" s="6"/>
+      <c r="AS5" s="6"/>
+      <c r="AT5" s="6"/>
+      <c r="AU5" s="6"/>
+      <c r="AV5" s="6"/>
+      <c r="AW5" s="6"/>
+      <c r="AX5" s="6"/>
+      <c r="AY5" s="6"/>
+      <c r="AZ5" s="6"/>
+      <c r="BA5" s="6"/>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:53" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
+      <c r="C6" s="8"/>
       <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
+      <c r="E6" s="8"/>
       <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
+      <c r="G6" s="8"/>
       <c r="H6" s="6"/>
-      <c r="I6" s="6"/>
-      <c r="J6" s="6"/>
-      <c r="K6" s="6"/>
-      <c r="L6" s="6"/>
-      <c r="M6" s="6"/>
-      <c r="N6" s="6"/>
-      <c r="O6" s="6"/>
-      <c r="P6" s="6"/>
-      <c r="Q6" s="6"/>
-      <c r="R6" s="6"/>
-      <c r="S6" s="6"/>
-      <c r="T6" s="6"/>
-      <c r="U6" s="6"/>
-      <c r="V6" s="6"/>
-      <c r="W6" s="6"/>
-      <c r="X6" s="6"/>
-      <c r="Y6" s="6"/>
-      <c r="Z6" s="6"/>
-      <c r="AA6" s="6"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
+      <c r="M6" s="8"/>
+      <c r="N6" s="8"/>
+      <c r="O6" s="8"/>
+      <c r="P6" s="8"/>
+      <c r="Q6" s="8"/>
+      <c r="R6" s="8"/>
+      <c r="S6" s="8"/>
+      <c r="T6" s="8"/>
+      <c r="U6" s="8"/>
+      <c r="V6" s="8"/>
+      <c r="W6" s="8"/>
+      <c r="X6" s="8"/>
+      <c r="Y6" s="8"/>
+      <c r="Z6" s="8"/>
+      <c r="AA6" s="8"/>
+      <c r="AB6" s="6"/>
+      <c r="AC6" s="6"/>
+      <c r="AD6" s="6"/>
+      <c r="AE6" s="6"/>
+      <c r="AF6" s="6"/>
+      <c r="AG6" s="6"/>
+      <c r="AH6" s="6"/>
+      <c r="AI6" s="6"/>
+      <c r="AJ6" s="6"/>
+      <c r="AK6" s="6"/>
+      <c r="AL6" s="6"/>
+      <c r="AM6" s="6"/>
+      <c r="AN6" s="6"/>
+      <c r="AO6" s="6"/>
+      <c r="AP6" s="6"/>
+      <c r="AQ6" s="6"/>
+      <c r="AR6" s="6"/>
+      <c r="AS6" s="6"/>
+      <c r="AT6" s="6"/>
+      <c r="AU6" s="6"/>
+      <c r="AV6" s="6"/>
+      <c r="AW6" s="6"/>
+      <c r="AX6" s="6"/>
+      <c r="AY6" s="6"/>
+      <c r="AZ6" s="6"/>
+      <c r="BA6" s="6"/>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A7" s="4" t="s">
+    <row r="7" spans="1:53" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="7"/>
+      <c r="N7" s="7"/>
+      <c r="O7" s="7"/>
+      <c r="P7" s="7"/>
+      <c r="Q7" s="7"/>
+      <c r="R7" s="7"/>
+      <c r="S7" s="7"/>
+      <c r="T7" s="7"/>
+      <c r="U7" s="7"/>
+      <c r="V7" s="7"/>
+      <c r="W7" s="7"/>
+      <c r="X7" s="7"/>
+      <c r="Y7" s="7"/>
+      <c r="Z7" s="7"/>
+      <c r="AA7" s="7"/>
+      <c r="AB7" s="6"/>
+      <c r="AC7" s="6"/>
+      <c r="AD7" s="6"/>
+      <c r="AE7" s="6"/>
+      <c r="AF7" s="6"/>
+      <c r="AG7" s="6"/>
+      <c r="AH7" s="6"/>
+      <c r="AI7" s="6"/>
+      <c r="AJ7" s="6"/>
+      <c r="AK7" s="6"/>
+      <c r="AL7" s="6"/>
+      <c r="AM7" s="6"/>
+      <c r="AN7" s="6"/>
+      <c r="AO7" s="6"/>
+      <c r="AP7" s="6"/>
+      <c r="AQ7" s="6"/>
+      <c r="AR7" s="6"/>
+      <c r="AS7" s="6"/>
+      <c r="AT7" s="6"/>
+      <c r="AU7" s="6"/>
+      <c r="AV7" s="6"/>
+      <c r="AW7" s="6"/>
+      <c r="AX7" s="6"/>
+      <c r="AY7" s="6"/>
+      <c r="AZ7" s="6"/>
+      <c r="BA7" s="6"/>
+    </row>
+    <row r="8" spans="1:53" x14ac:dyDescent="0.2">
+      <c r="A8" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="6"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6"/>
-      <c r="M7" s="6"/>
-      <c r="N7" s="6"/>
-      <c r="O7" s="6"/>
-      <c r="P7" s="6"/>
-      <c r="Q7" s="6"/>
-      <c r="R7" s="6"/>
-      <c r="S7" s="6"/>
-      <c r="T7" s="6"/>
-      <c r="U7" s="6"/>
-      <c r="V7" s="6"/>
-      <c r="W7" s="6"/>
-      <c r="X7" s="6"/>
-      <c r="Y7" s="6"/>
-      <c r="Z7" s="6"/>
-      <c r="AA7" s="6"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="9"/>
+      <c r="J8" s="9"/>
+      <c r="K8" s="9"/>
+      <c r="L8" s="9"/>
+      <c r="M8" s="9"/>
+      <c r="N8" s="9"/>
+      <c r="O8" s="9"/>
+      <c r="P8" s="9"/>
+      <c r="Q8" s="9"/>
+      <c r="R8" s="9"/>
+      <c r="S8" s="9"/>
+      <c r="T8" s="9"/>
+      <c r="U8" s="9"/>
+      <c r="V8" s="9"/>
+      <c r="W8" s="9"/>
+      <c r="X8" s="9"/>
+      <c r="Y8" s="9"/>
+      <c r="Z8" s="9"/>
+      <c r="AA8" s="9"/>
+      <c r="AB8" s="6"/>
+      <c r="AC8" s="6"/>
+      <c r="AD8" s="6"/>
+      <c r="AE8" s="6"/>
+      <c r="AF8" s="6"/>
+      <c r="AG8" s="6"/>
+      <c r="AH8" s="6"/>
+      <c r="AI8" s="6"/>
+      <c r="AJ8" s="6"/>
+      <c r="AK8" s="6"/>
+      <c r="AL8" s="6"/>
+      <c r="AM8" s="6"/>
+      <c r="AN8" s="6"/>
+      <c r="AO8" s="6"/>
+      <c r="AP8" s="6"/>
+      <c r="AQ8" s="6"/>
+      <c r="AR8" s="6"/>
+      <c r="AS8" s="6"/>
+      <c r="AT8" s="6"/>
+      <c r="AU8" s="6"/>
+      <c r="AV8" s="6"/>
+      <c r="AW8" s="6"/>
+      <c r="AX8" s="6"/>
+      <c r="AY8" s="6"/>
+      <c r="AZ8" s="6"/>
+      <c r="BA8" s="6"/>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A8" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="6"/>
-      <c r="J8" s="6"/>
-      <c r="K8" s="6"/>
-      <c r="L8" s="6"/>
-      <c r="M8" s="6"/>
-      <c r="N8" s="6"/>
-      <c r="O8" s="6"/>
-      <c r="P8" s="6"/>
-      <c r="Q8" s="6"/>
-      <c r="R8" s="6"/>
-      <c r="S8" s="6"/>
-      <c r="T8" s="6"/>
-      <c r="U8" s="6"/>
-      <c r="V8" s="6"/>
-      <c r="W8" s="6"/>
-      <c r="X8" s="6"/>
-      <c r="Y8" s="6"/>
-      <c r="Z8" s="6"/>
-      <c r="AA8" s="6"/>
+    <row r="9" spans="1:53" x14ac:dyDescent="0.2">
+      <c r="A9" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="6"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="9"/>
+      <c r="J9" s="9"/>
+      <c r="K9" s="9"/>
+      <c r="L9" s="9"/>
+      <c r="M9" s="9"/>
+      <c r="N9" s="9"/>
+      <c r="O9" s="9"/>
+      <c r="P9" s="9"/>
+      <c r="Q9" s="9"/>
+      <c r="R9" s="9"/>
+      <c r="S9" s="9"/>
+      <c r="T9" s="9"/>
+      <c r="U9" s="9"/>
+      <c r="V9" s="9"/>
+      <c r="W9" s="9"/>
+      <c r="X9" s="9"/>
+      <c r="Y9" s="9"/>
+      <c r="Z9" s="9"/>
+      <c r="AA9" s="9"/>
+      <c r="AB9" s="6"/>
+      <c r="AC9" s="6"/>
+      <c r="AD9" s="6"/>
+      <c r="AE9" s="6"/>
+      <c r="AF9" s="6"/>
+      <c r="AG9" s="6"/>
+      <c r="AH9" s="6"/>
+      <c r="AI9" s="6"/>
+      <c r="AJ9" s="6"/>
+      <c r="AK9" s="6"/>
+      <c r="AL9" s="6"/>
+      <c r="AM9" s="6"/>
+      <c r="AN9" s="6"/>
+      <c r="AO9" s="6"/>
+      <c r="AP9" s="6"/>
+      <c r="AQ9" s="6"/>
+      <c r="AR9" s="6"/>
+      <c r="AS9" s="6"/>
+      <c r="AT9" s="6"/>
+      <c r="AU9" s="6"/>
+      <c r="AV9" s="6"/>
+      <c r="AW9" s="6"/>
+      <c r="AX9" s="6"/>
+      <c r="AY9" s="6"/>
+      <c r="AZ9" s="6"/>
+      <c r="BA9" s="6"/>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="6"/>
-      <c r="J9" s="6"/>
-      <c r="K9" s="6"/>
-      <c r="L9" s="6"/>
-      <c r="M9" s="6"/>
-      <c r="N9" s="6"/>
-      <c r="O9" s="6"/>
-      <c r="P9" s="6"/>
-      <c r="Q9" s="6"/>
-      <c r="R9" s="6"/>
-      <c r="S9" s="6"/>
-      <c r="T9" s="6"/>
-      <c r="U9" s="6"/>
-      <c r="V9" s="6"/>
-      <c r="W9" s="6"/>
-      <c r="X9" s="6"/>
-      <c r="Y9" s="6"/>
-      <c r="Z9" s="6"/>
-      <c r="AA9" s="6"/>
+    <row r="10" spans="1:53" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" t="s">
+        <v>2</v>
+      </c>
+      <c r="C10" t="s">
+        <v>6</v>
+      </c>
+      <c r="D10" t="s">
+        <v>2</v>
+      </c>
+      <c r="E10" t="s">
+        <v>6</v>
+      </c>
+      <c r="F10" t="s">
+        <v>2</v>
+      </c>
+      <c r="G10" t="s">
+        <v>6</v>
+      </c>
+      <c r="H10" t="s">
+        <v>2</v>
+      </c>
+      <c r="I10" t="s">
+        <v>6</v>
+      </c>
+      <c r="J10" t="s">
+        <v>2</v>
+      </c>
+      <c r="K10" t="s">
+        <v>6</v>
+      </c>
+      <c r="L10" t="s">
+        <v>2</v>
+      </c>
+      <c r="M10" t="s">
+        <v>6</v>
+      </c>
+      <c r="N10" t="s">
+        <v>2</v>
+      </c>
+      <c r="O10" t="s">
+        <v>6</v>
+      </c>
+      <c r="P10" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>6</v>
+      </c>
+      <c r="R10" t="s">
+        <v>2</v>
+      </c>
+      <c r="S10" t="s">
+        <v>6</v>
+      </c>
+      <c r="T10" t="s">
+        <v>2</v>
+      </c>
+      <c r="U10" t="s">
+        <v>6</v>
+      </c>
+      <c r="V10" t="s">
+        <v>2</v>
+      </c>
+      <c r="W10" t="s">
+        <v>6</v>
+      </c>
+      <c r="X10" t="s">
+        <v>2</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>6</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>2</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>6</v>
+      </c>
+      <c r="AB10" t="s">
+        <v>2</v>
+      </c>
+      <c r="AC10" t="s">
+        <v>6</v>
+      </c>
+      <c r="AD10" t="s">
+        <v>2</v>
+      </c>
+      <c r="AE10" t="s">
+        <v>6</v>
+      </c>
+      <c r="AF10" t="s">
+        <v>2</v>
+      </c>
+      <c r="AG10" t="s">
+        <v>6</v>
+      </c>
+      <c r="AH10" t="s">
+        <v>2</v>
+      </c>
+      <c r="AI10" t="s">
+        <v>6</v>
+      </c>
+      <c r="AJ10" t="s">
+        <v>2</v>
+      </c>
+      <c r="AK10" t="s">
+        <v>6</v>
+      </c>
+      <c r="AL10" t="s">
+        <v>2</v>
+      </c>
+      <c r="AM10" t="s">
+        <v>6</v>
+      </c>
+      <c r="AN10" t="s">
+        <v>2</v>
+      </c>
+      <c r="AO10" t="s">
+        <v>6</v>
+      </c>
+      <c r="AP10" t="s">
+        <v>2</v>
+      </c>
+      <c r="AQ10" t="s">
+        <v>6</v>
+      </c>
+      <c r="AR10" t="s">
+        <v>2</v>
+      </c>
+      <c r="AS10" t="s">
+        <v>6</v>
+      </c>
+      <c r="AT10" t="s">
+        <v>2</v>
+      </c>
+      <c r="AU10" t="s">
+        <v>6</v>
+      </c>
+      <c r="AV10" t="s">
+        <v>2</v>
+      </c>
+      <c r="AW10" t="s">
+        <v>6</v>
+      </c>
+      <c r="AX10" t="s">
+        <v>2</v>
+      </c>
+      <c r="AY10" t="s">
+        <v>6</v>
+      </c>
+      <c r="AZ10" t="s">
+        <v>2</v>
+      </c>
+      <c r="BA10" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A10" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="6"/>
-      <c r="M10" s="6"/>
-      <c r="N10" s="6"/>
-      <c r="O10" s="6"/>
-      <c r="P10" s="6"/>
-      <c r="Q10" s="6"/>
-      <c r="R10" s="6"/>
-      <c r="S10" s="6"/>
-      <c r="T10" s="6"/>
-      <c r="U10" s="6"/>
-      <c r="V10" s="6"/>
-      <c r="W10" s="6"/>
-      <c r="X10" s="6"/>
-      <c r="Y10" s="6"/>
-      <c r="Z10" s="6"/>
-      <c r="AA10" s="6"/>
+    <row r="14" spans="1:53" x14ac:dyDescent="0.2">
+      <c r="A14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+      <c r="O14" s="1"/>
+      <c r="P14" s="1"/>
+      <c r="Q14" s="1"/>
+      <c r="R14" s="1"/>
+      <c r="S14" s="1"/>
+      <c r="T14" s="1"/>
+      <c r="U14" s="1"/>
+      <c r="V14" s="1"/>
+      <c r="W14" s="1"/>
+      <c r="X14" s="1"/>
+      <c r="Y14" s="1"/>
+      <c r="Z14" s="1"/>
+      <c r="AA14" s="1"/>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A11" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="6"/>
-      <c r="M11" s="6"/>
-      <c r="N11" s="6"/>
-      <c r="O11" s="6"/>
-      <c r="P11" s="6"/>
-      <c r="Q11" s="6"/>
-      <c r="R11" s="6"/>
-      <c r="S11" s="6"/>
-      <c r="T11" s="6"/>
-      <c r="U11" s="6"/>
-      <c r="V11" s="6"/>
-      <c r="W11" s="6"/>
-      <c r="X11" s="6"/>
-      <c r="Y11" s="6"/>
-      <c r="Z11" s="6"/>
-      <c r="AA11" s="6"/>
+    <row r="15" spans="1:53" x14ac:dyDescent="0.2">
+      <c r="A15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1"/>
+      <c r="K15" s="1"/>
+      <c r="L15" s="1"/>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
+      <c r="O15" s="1"/>
+      <c r="P15" s="1"/>
+      <c r="Q15" s="1"/>
+      <c r="R15" s="1"/>
+      <c r="S15" s="1"/>
+      <c r="T15" s="1"/>
+      <c r="U15" s="1"/>
+      <c r="V15" s="1"/>
+      <c r="W15" s="1"/>
+      <c r="X15" s="1"/>
+      <c r="Y15" s="1"/>
+      <c r="Z15" s="1"/>
+      <c r="AA15" s="1"/>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:53" x14ac:dyDescent="0.2">
       <c r="A16" s="1"/>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" s="1"/>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+      <c r="O16" s="1"/>
+      <c r="P16" s="1"/>
+      <c r="Q16" s="1"/>
+      <c r="R16" s="1"/>
+      <c r="S16" s="1"/>
+      <c r="T16" s="1"/>
+      <c r="U16" s="1"/>
+      <c r="V16" s="1"/>
+      <c r="W16" s="1"/>
+      <c r="X16" s="1"/>
+      <c r="Y16" s="1"/>
+      <c r="Z16" s="1"/>
+      <c r="AA16" s="1"/>
     </row>
   </sheetData>
+  <mergeCells count="26">
+    <mergeCell ref="AX1:AY1"/>
+    <mergeCell ref="AZ1:BA1"/>
+    <mergeCell ref="AL1:AM1"/>
+    <mergeCell ref="AN1:AO1"/>
+    <mergeCell ref="AP1:AQ1"/>
+    <mergeCell ref="AR1:AS1"/>
+    <mergeCell ref="AT1:AU1"/>
+    <mergeCell ref="AV1:AW1"/>
+    <mergeCell ref="Z1:AA1"/>
+    <mergeCell ref="AB1:AC1"/>
+    <mergeCell ref="AD1:AE1"/>
+    <mergeCell ref="AF1:AG1"/>
+    <mergeCell ref="AH1:AI1"/>
+    <mergeCell ref="AJ1:AK1"/>
+    <mergeCell ref="N1:O1"/>
+    <mergeCell ref="P1:Q1"/>
+    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="T1:U1"/>
+    <mergeCell ref="V1:W1"/>
+    <mergeCell ref="X1:Y1"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="L1:M1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>